<commit_message>
Wrote script for Login Functionality for TC_LF_003, TC_LF_004 cases
</commit_message>
<xml_diff>
--- a/manual_test_cases/Daraz_Manual_Test_Checklist.xlsx
+++ b/manual_test_cases/Daraz_Manual_Test_Checklist.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shifa\OneDrive\Documents\Manual Projects\Daraz\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\Automation_project\Daraz_Website_Automation_Using_Playwright\manual_test_cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51CAC49F-6DC0-463B-936E-57B1F132A9D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E224BF2E-348F-4706-8C7A-AFD70BD55B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-12675" windowWidth="29040" windowHeight="15720" xr2:uid="{02469D76-9D46-4AA2-AC21-F8D260897AAE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{02469D76-9D46-4AA2-AC21-F8D260897AAE}"/>
   </bookViews>
   <sheets>
     <sheet name="Version History" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="436">
   <si>
     <t>Project Name :</t>
   </si>
@@ -457,65 +457,15 @@
     <t>Warning message is not displayed. The user is successfully logged in using an invalid password.</t>
   </si>
   <si>
-    <t xml:space="preserve">Email address : xabcdrt@gmail.com
-Phone number : +918376592
-Password : abcdeg$ </t>
-  </si>
-  <si>
     <t xml:space="preserve">Not Applicable </t>
   </si>
   <si>
     <t>Validate 'Forgotten Password' link is available in the login page and working properly.</t>
-  </si>
-  <si>
-    <r>
-      <t>1) Click on 'Login' option.
-2) Click on 'Forgotten Password' link. (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>*</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>)</t>
-    </r>
   </si>
   <si>
     <t>1) Click on 'Login' option.
 2) Enter registered mobile number in the 'Phone Number' filed.
 3) Enter valid password in the 'Password' filed.
-4) Click on 'Continue' button.</t>
-  </si>
-  <si>
-    <t>1) Click on 'Login' option.
-2) Enter invalid email address in the 'Email Address' filed or invalid phone number in the 'Phone number' field.
-3) Enter valid password in the 'Password' filed.
-4) Click on 'Continue' button.</t>
-  </si>
-  <si>
-    <t>1) Click on 'Login' option.
-2) Enter valid email address in the 'Email Address' filed or valid phone number in the 'Phone number' field.
-3) Enter invalid password in the 'Password' filed.
-4) Click on 'Continue' button.</t>
-  </si>
-  <si>
-    <t>1) Click on 'Login' option.
-2) Enter invalid email address in the 'Email Address' filed or invalid phone number in the 'Phone number' field.
-3) Enter invalid password in the 'Password' filed.
 4) Click on 'Continue' button.</t>
   </si>
   <si>
@@ -553,18 +503,6 @@
 2) Enter a valid email address in the 'Email Address' field.
 3) Enter valid password in the 'Password' filed.
 4) Click on 'Continue' button.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validate login to the application using invalid credentials. 
-(i.e., Invalid email address or invalid mobile number) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validate login to the application using invalid credentials. 
-(i.e., Invalid password) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validate login to the application using invalid credentials. 
-(i.e., Invalid email address or invalid mobile number and invalid password) </t>
   </si>
   <si>
     <t xml:space="preserve">Validate login to the application without providing any credentials. </t>
@@ -1686,59 +1624,6 @@
         <scheme val="minor"/>
       </rPr>
       <t>!').
-• The user should remain on the login page.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>•</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16.100000000000001"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>The system should not allow the user to log in with invalid credentials.
-• An appropriate error message should be displayed (e.g., '</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Invalid Email Address or Invalid Phone Number and/or Invalid Password !</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>').
 • The user should remain on the login page.</t>
     </r>
   </si>
@@ -2764,6 +2649,152 @@
   </si>
   <si>
     <t xml:space="preserve"> Md. Shifat Laskor &amp; Md. Hasibur Rahman</t>
+  </si>
+  <si>
+    <t>1) Click on 'Login' option.
+2) Enter invalid email address in the 'Email Address' filed.
+3) Enter valid password in the 'Password' filed.
+4) Click on 'Continue' button.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email address : xabcdrt@gmail.com
+Password : Daraz1234$ </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>•</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16.100000000000001"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The system should not allow the user to log in with invalid credentials.
+• An appropriate error message should be displayed (e.g.,  '</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Invalid account or password</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>').
+• The user should remain on the login page.</t>
+    </r>
+  </si>
+  <si>
+    <t>1) Click on 'Login' option.
+2) Enter valid email address in the 'Email Address' filed.
+3) Enter invalid password in the 'Password' filed.
+4) Click on 'Continue' button.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validate login to the application using invalid credentials. 
+(i.e., Invalid email address and invalid password) </t>
+  </si>
+  <si>
+    <t>1) Click on 'Login' option.
+2) Enter invalid email address in the 'Email Address' filed.
+3) Enter invalid password in the 'Password' filed. 
+4) Click on 'Continue' button.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email address : abcd@gmail.com
+Password : abcd$ </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>•</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16.100000000000001"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The system should not allow the user to log in with invalid credentials.
+• An appropriate message should be displayed under the input box (e.g., '</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>You can't leave this field empty</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>').
+• The user should remain on the login page.</t>
+    </r>
+  </si>
+  <si>
+    <t>1) Click on 'Login' option.
+2) Click on 'Forgotten Password' link.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validate login to the application using invalid credentials (Invalid email address and valid password) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validate login to the application using  invalid credentials (valid email address and invalid password) </t>
   </si>
 </sst>
 </file>
@@ -2908,7 +2939,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2984,6 +3015,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3001,9 +3035,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3330,21 +3361,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1122DB24-336C-4BDE-AAFD-8F064C42F5B9}">
   <dimension ref="G1:U7"/>
-  <sheetFormatPr defaultRowHeight="26.25" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="25.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="7" max="7" width="45.85546875" style="17" customWidth="1"/>
-    <col min="8" max="8" width="2.140625" customWidth="1"/>
-    <col min="9" max="9" width="45.85546875" style="14" customWidth="1"/>
+    <col min="7" max="7" width="45.88671875" style="17" customWidth="1"/>
+    <col min="8" max="8" width="2.109375" customWidth="1"/>
+    <col min="9" max="9" width="45.88671875" style="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="7:21" ht="23.45" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="7:21" ht="60.6" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="7:21" ht="23.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="7:21" ht="60.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="G2" s="18" t="s">
         <v>0</v>
       </c>
       <c r="H2" s="16"/>
       <c r="I2" s="15" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="O2" s="19"/>
       <c r="P2" s="19"/>
@@ -3354,13 +3385,13 @@
       <c r="T2" s="20"/>
       <c r="U2" s="20"/>
     </row>
-    <row r="3" spans="7:21" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="7:21" ht="60" customHeight="1" x14ac:dyDescent="0.4">
       <c r="G3" s="18" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="16"/>
-      <c r="I3" s="30" t="s">
-        <v>433</v>
+      <c r="I3" s="22" t="s">
+        <v>424</v>
       </c>
       <c r="O3" s="19"/>
       <c r="P3" s="19"/>
@@ -3370,13 +3401,13 @@
       <c r="T3" s="20"/>
       <c r="U3" s="20"/>
     </row>
-    <row r="4" spans="7:21" ht="60.6" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="7:21" ht="60.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="G4" s="18" t="s">
         <v>1</v>
       </c>
       <c r="H4" s="16"/>
       <c r="I4" s="15" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="O4" s="19"/>
       <c r="P4" s="19"/>
@@ -3386,9 +3417,9 @@
       <c r="T4" s="20"/>
       <c r="U4" s="20"/>
     </row>
-    <row r="5" spans="7:21" ht="44.45" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="7:21" ht="55.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="7:21" ht="55.9" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="7:21" ht="44.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="7:21" ht="55.2" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="7:21" ht="55.95" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3398,33 +3429,33 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0792B093-2DBC-41B2-A40D-647FCC4C9792}">
   <dimension ref="A1:J16"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="2" width="20.85546875" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" customWidth="1"/>
-    <col min="4" max="4" width="40.85546875" style="11" customWidth="1"/>
-    <col min="5" max="5" width="71.140625" customWidth="1"/>
-    <col min="6" max="6" width="48.140625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="57.42578125" customWidth="1"/>
-    <col min="8" max="8" width="51.5703125" customWidth="1"/>
-    <col min="9" max="10" width="25.7109375" style="11" customWidth="1"/>
+    <col min="1" max="2" width="20.88671875" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" customWidth="1"/>
+    <col min="4" max="4" width="40.88671875" style="11" customWidth="1"/>
+    <col min="5" max="5" width="71.109375" customWidth="1"/>
+    <col min="6" max="6" width="48.109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="57.44140625" customWidth="1"/>
+    <col min="8" max="8" width="51.5546875" customWidth="1"/>
+    <col min="9" max="10" width="25.6640625" style="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>343</v>
+        <v>334</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>344</v>
+        <v>335</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>362</v>
+        <v>353</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>345</v>
+        <v>336</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>67</v>
@@ -3436,13 +3467,13 @@
         <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="6"/>
@@ -3453,56 +3484,56 @@
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
     </row>
-    <row r="3" spans="1:10" ht="152.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="152.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>348</v>
+        <v>339</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>363</v>
+        <v>354</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>364</v>
+        <v>355</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>366</v>
+        <v>357</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
       <c r="H3" s="7" t="s">
         <v>34</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>367</v>
+        <v>358</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" s="1" customFormat="1" ht="143.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" s="1" customFormat="1" ht="143.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>349</v>
+        <v>340</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>371</v>
+        <v>362</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>372</v>
+        <v>363</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>75</v>
@@ -3511,394 +3542,394 @@
         <v>40</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>367</v>
+        <v>358</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="155.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="155.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>350</v>
+        <v>341</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>59</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>373</v>
+        <v>364</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>56</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>71</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="H5" s="7" t="s">
         <v>72</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>367</v>
+        <v>358</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="139.15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="139.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>351</v>
+        <v>342</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>60</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>375</v>
+        <v>366</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>56</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>378</v>
+        <v>369</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>381</v>
+        <v>372</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>78</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>367</v>
+        <v>358</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="159" customHeight="1" x14ac:dyDescent="0.25">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="159" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>352</v>
+        <v>343</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>377</v>
+        <v>368</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>77</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>383</v>
+        <v>374</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>353</v>
+        <v>344</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>385</v>
+        <v>376</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>386</v>
+        <v>377</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>77</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>387</v>
+        <v>378</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>388</v>
+        <v>379</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>383</v>
+        <v>374</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="168.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="168.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>354</v>
+        <v>345</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>389</v>
+        <v>380</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>77</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="I9" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="193.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>383</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>391</v>
       </c>
-      <c r="J9" s="4" t="s">
+      <c r="G10" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="I10" s="4" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" ht="193.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>392</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>399</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>400</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>401</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>383</v>
-      </c>
       <c r="J10" s="4" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.25">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>356</v>
+        <v>347</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>403</v>
+        <v>394</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>77</v>
       </c>
       <c r="G11" s="7" t="s">
+        <v>396</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="256.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>398</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="270" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>401</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>404</v>
+      </c>
+      <c r="F13" s="5" t="s">
         <v>405</v>
       </c>
-      <c r="H11" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>383</v>
-      </c>
-      <c r="J11" s="4" t="s">
+      <c r="G13" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="264.60000000000002" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>406</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" ht="256.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>357</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="C12" s="7" t="s">
+      <c r="D14" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="E14" s="7" t="s">
         <v>407</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="E12" s="7" t="s">
+      <c r="F14" s="5" t="s">
         <v>408</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="G14" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="292.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>409</v>
       </c>
-      <c r="G12" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>391</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="270" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>358</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="C13" s="5" t="s">
+      <c r="D15" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="E15" s="7" t="s">
         <v>410</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="E13" s="7" t="s">
+      <c r="F15" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="271.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>413</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="D16" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="E16" s="7" t="s">
         <v>414</v>
       </c>
-      <c r="G13" s="7" t="s">
-        <v>412</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>258</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>391</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="264.60000000000002" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>359</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="C14" s="7" t="s">
+      <c r="F16" s="5" t="s">
         <v>415</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>416</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>326</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>367</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="292.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>360</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>418</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>282</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>419</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>294</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>295</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>391</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="271.89999999999998" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>361</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>282</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>423</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>424</v>
-      </c>
       <c r="G16" s="7" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>391</v>
+        <v>382</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>374</v>
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -3911,21 +3942,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{160DC5CE-D4D6-45E5-9673-C5134C0EE041}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
-    <col min="3" max="3" width="45.85546875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="70.85546875" style="7" customWidth="1"/>
-    <col min="5" max="5" width="48.140625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="70.7109375" style="7" customWidth="1"/>
-    <col min="7" max="7" width="71.5703125" style="7" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="4" customWidth="1"/>
+    <col min="1" max="1" width="21.44140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" customWidth="1"/>
+    <col min="3" max="3" width="45.88671875" style="6" customWidth="1"/>
+    <col min="4" max="4" width="70.88671875" style="7" customWidth="1"/>
+    <col min="5" max="5" width="48.109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="70.6640625" style="7" customWidth="1"/>
+    <col min="7" max="7" width="71.5546875" style="7" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="4" customWidth="1"/>
     <col min="9" max="9" width="26" style="4" customWidth="1"/>
-    <col min="10" max="10" width="14.85546875" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -3954,33 +3985,33 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="28" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
-        <v>429</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>428</v>
-      </c>
-      <c r="C3" s="24" t="s">
-        <v>430</v>
-      </c>
-      <c r="D3" s="25" t="s">
-        <v>425</v>
-      </c>
-      <c r="E3" s="24" t="s">
-        <v>426</v>
-      </c>
-      <c r="F3" s="25" t="s">
-        <v>427</v>
-      </c>
-      <c r="G3" s="25" t="s">
+    <row r="3" spans="1:10" s="29" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="23" t="s">
+        <v>420</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>419</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>421</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>416</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>417</v>
+      </c>
+      <c r="F3" s="26" t="s">
+        <v>418</v>
+      </c>
+      <c r="G3" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="H3" s="23" t="s">
+      <c r="H3" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="26"/>
-      <c r="J3" s="27"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3991,20 +4022,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{126F3227-500D-408C-A3D2-9A52BE2F4C8C}">
   <dimension ref="A1:I31"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
-    <col min="3" max="3" width="45.85546875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="70.85546875" style="7" customWidth="1"/>
-    <col min="5" max="5" width="48.140625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="70.7109375" style="7" customWidth="1"/>
-    <col min="7" max="7" width="71.5703125" style="7" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="4" customWidth="1"/>
+    <col min="1" max="1" width="21.44140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" customWidth="1"/>
+    <col min="3" max="3" width="45.88671875" style="6" customWidth="1"/>
+    <col min="4" max="4" width="70.88671875" style="7" customWidth="1"/>
+    <col min="5" max="5" width="48.109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="70.6640625" style="7" customWidth="1"/>
+    <col min="7" max="7" width="71.5546875" style="7" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="4" customWidth="1"/>
     <col min="9" max="9" width="26" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -4033,7 +4064,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="156.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="156.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
@@ -4044,10 +4075,10 @@
         <v>24</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>365</v>
+        <v>356</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>336</v>
+        <v>327</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>20</v>
@@ -4062,7 +4093,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="1" customFormat="1" ht="150" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="1" customFormat="1" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
@@ -4073,13 +4104,13 @@
         <v>26</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>333</v>
+        <v>324</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>369</v>
+        <v>360</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>34</v>
@@ -4091,7 +4122,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="154.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="154.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
@@ -4102,10 +4133,10 @@
         <v>29</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>334</v>
+        <v>325</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>73</v>
@@ -4120,7 +4151,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="117.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="117.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
@@ -4134,7 +4165,7 @@
         <v>31</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>335</v>
+        <v>326</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>32</v>
@@ -4149,7 +4180,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="157.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="157.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>13</v>
       </c>
@@ -4163,7 +4194,7 @@
         <v>38</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>74</v>
@@ -4178,7 +4209,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="165" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="165" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
@@ -4192,7 +4223,7 @@
         <v>39</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>75</v>
@@ -4207,7 +4238,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="128.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="128.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>15</v>
       </c>
@@ -4221,7 +4252,7 @@
         <v>43</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="F9" s="7" t="s">
         <v>44</v>
@@ -4236,7 +4267,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="178.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="178.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>16</v>
       </c>
@@ -4250,7 +4281,7 @@
         <v>46</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>47</v>
@@ -4265,7 +4296,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="165.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="165.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>17</v>
       </c>
@@ -4279,7 +4310,7 @@
         <v>50</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>336</v>
+        <v>327</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>76</v>
@@ -4294,7 +4325,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="120.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="120.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>18</v>
       </c>
@@ -4308,7 +4339,7 @@
         <v>52</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>335</v>
+        <v>326</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>53</v>
@@ -4323,7 +4354,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="120.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="120.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>18</v>
       </c>
@@ -4337,7 +4368,7 @@
         <v>52</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>335</v>
+        <v>326</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>53</v>
@@ -4352,25 +4383,25 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C25" s="21"/>
     </row>
-    <row r="26" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C26" s="21"/>
     </row>
-    <row r="27" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C27" s="21"/>
     </row>
-    <row r="28" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C28" s="21"/>
     </row>
-    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C29" s="21"/>
     </row>
-    <row r="30" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C30" s="21"/>
     </row>
-    <row r="31" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C31" s="21"/>
     </row>
   </sheetData>
@@ -4383,20 +4414,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E58948E-B793-4546-A904-38FBA4A9768B}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" customWidth="1"/>
-    <col min="4" max="4" width="71.140625" customWidth="1"/>
-    <col min="5" max="5" width="40.85546875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="62.85546875" customWidth="1"/>
-    <col min="7" max="7" width="43.5703125" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="11" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" customWidth="1"/>
+    <col min="4" max="4" width="71.109375" customWidth="1"/>
+    <col min="5" max="5" width="40.88671875" style="11" customWidth="1"/>
+    <col min="6" max="6" width="62.88671875" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="11" customWidth="1"/>
     <col min="9" max="9" width="26" style="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -4425,7 +4456,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="C2" s="6"/>
       <c r="D2" s="7"/>
@@ -4435,123 +4466,123 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" s="28" customFormat="1" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+    <row r="3" spans="1:9" s="29" customFormat="1" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="24" t="s">
-        <v>431</v>
-      </c>
-      <c r="D3" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="E3" s="24" t="s">
+      <c r="C3" s="25" t="s">
+        <v>422</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>81</v>
+      </c>
+      <c r="E3" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="F3" s="25" t="s">
+      <c r="F3" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="G3" s="25" t="s">
+      <c r="G3" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="H3" s="23" t="s">
+      <c r="H3" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="23" t="s">
+      <c r="I3" s="24" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="29" customFormat="1" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="22" t="s">
+    <row r="4" spans="1:9" s="30" customFormat="1" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="C4" s="24" t="s">
-        <v>432</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>94</v>
-      </c>
-      <c r="E4" s="24" t="s">
+      <c r="C4" s="25" t="s">
+        <v>423</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="F4" s="25" t="s">
+      <c r="F4" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="G4" s="25" t="s">
+      <c r="G4" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="H4" s="23" t="s">
+      <c r="H4" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="23" t="s">
+      <c r="I4" s="24" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="105.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:9" s="29" customFormat="1" ht="105.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>318</v>
-      </c>
-      <c r="G5" s="7" t="s">
+      <c r="C5" s="25" t="s">
+        <v>434</v>
+      </c>
+      <c r="D5" s="26" t="s">
+        <v>425</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>426</v>
+      </c>
+      <c r="F5" s="26" t="s">
+        <v>427</v>
+      </c>
+      <c r="G5" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="13" t="s">
+      <c r="I5" s="24" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="29" customFormat="1" ht="109.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>435</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>428</v>
+      </c>
+      <c r="E6" s="25" t="s">
+        <v>367</v>
+      </c>
+      <c r="F6" s="26" t="s">
+        <v>427</v>
+      </c>
+      <c r="G6" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="H6" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="24" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="109.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>376</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>319</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="I6" s="13" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="136.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="136.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>61</v>
       </c>
@@ -4559,16 +4590,16 @@
         <v>56</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>97</v>
+        <v>429</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>86</v>
+        <v>430</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>79</v>
+        <v>431</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>320</v>
+        <v>427</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>33</v>
@@ -4580,7 +4611,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="136.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="118.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>62</v>
       </c>
@@ -4588,16 +4619,16 @@
         <v>56</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>320</v>
+        <v>432</v>
       </c>
       <c r="G8" s="7" t="s">
         <v>33</v>
@@ -4609,7 +4640,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="116.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>63</v>
       </c>
@@ -4617,19 +4648,19 @@
         <v>56</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>82</v>
+        <v>433</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>27</v>
@@ -4638,7 +4669,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="126.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="126.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>64</v>
       </c>
@@ -4646,16 +4677,16 @@
         <v>56</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>77</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>33</v>
@@ -4667,7 +4698,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="125.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="125.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>65</v>
       </c>
@@ -4675,19 +4706,19 @@
         <v>56</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>77</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>54</v>
@@ -4696,7 +4727,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="140.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="140.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>66</v>
       </c>
@@ -4704,16 +4735,16 @@
         <v>56</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>77</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>33</v>
@@ -4735,20 +4766,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B70680C-BD57-41BD-B550-973B32609FA9}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" customWidth="1"/>
-    <col min="4" max="4" width="71.140625" customWidth="1"/>
-    <col min="5" max="5" width="40.85546875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="62.85546875" customWidth="1"/>
-    <col min="7" max="7" width="43.5703125" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="11" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" customWidth="1"/>
+    <col min="4" max="4" width="71.109375" customWidth="1"/>
+    <col min="5" max="5" width="40.88671875" style="11" customWidth="1"/>
+    <col min="6" max="6" width="62.88671875" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="11" customWidth="1"/>
     <col min="9" max="9" width="26" style="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -4777,7 +4808,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="C2" s="6"/>
       <c r="D2" s="7"/>
@@ -4787,24 +4818,24 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="100.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>123</v>
-      </c>
       <c r="E3" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>33</v>
@@ -4816,27 +4847,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="1" customFormat="1" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="1" customFormat="1" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>27</v>
@@ -4845,24 +4876,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="100.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>114</v>
-      </c>
       <c r="C5" s="5" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>33</v>
@@ -4874,24 +4905,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>122</v>
-      </c>
       <c r="E6" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>33</v>
@@ -4903,24 +4934,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="100.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>33</v>
@@ -4932,24 +4963,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="G8" s="7" t="s">
         <v>33</v>
@@ -4961,27 +4992,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="D9" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="F9" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="E9" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>138</v>
-      </c>
       <c r="G9" s="7" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>27</v>
@@ -4990,27 +5021,27 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>27</v>
@@ -5019,24 +5050,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>33</v>
@@ -5048,24 +5079,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="131.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="131.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>33</v>
@@ -5087,20 +5118,20 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0658FF2-697D-4C69-B42D-CDE2007A7D77}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" customWidth="1"/>
-    <col min="4" max="4" width="71.140625" customWidth="1"/>
-    <col min="5" max="5" width="40.85546875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="62.85546875" customWidth="1"/>
-    <col min="7" max="7" width="43.5703125" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="11" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" customWidth="1"/>
+    <col min="4" max="4" width="71.109375" customWidth="1"/>
+    <col min="5" max="5" width="40.88671875" style="11" customWidth="1"/>
+    <col min="6" max="6" width="62.88671875" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="11" customWidth="1"/>
     <col min="9" max="9" width="26" style="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -5129,7 +5160,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="C2" s="6"/>
       <c r="D2" s="7"/>
@@ -5139,24 +5170,24 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>70</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>33</v>
@@ -5168,27 +5199,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="1" customFormat="1" ht="90.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="1" customFormat="1" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>27</v>
@@ -5197,24 +5228,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>393</v>
+        <v>384</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>33</v>
@@ -5226,27 +5257,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>394</v>
+        <v>385</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>322</v>
+        <v>313</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>27</v>
@@ -5255,24 +5286,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>393</v>
+        <v>384</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>33</v>
@@ -5284,27 +5315,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>393</v>
+        <v>384</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>27</v>
@@ -5313,24 +5344,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="91.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="91.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>395</v>
+        <v>386</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>33</v>
@@ -5342,24 +5373,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="150" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>396</v>
+        <v>387</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>33</v>
@@ -5371,24 +5402,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>33</v>
@@ -5400,27 +5431,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>398</v>
+        <v>389</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>27</v>
@@ -5439,20 +5470,20 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B3B9881-CF40-4798-A105-6C45CF8840BD}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" customWidth="1"/>
-    <col min="4" max="4" width="71.140625" customWidth="1"/>
-    <col min="5" max="5" width="40.85546875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="62.85546875" customWidth="1"/>
-    <col min="7" max="7" width="43.5703125" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="11" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" customWidth="1"/>
+    <col min="4" max="4" width="71.109375" customWidth="1"/>
+    <col min="5" max="5" width="40.88671875" style="11" customWidth="1"/>
+    <col min="6" max="6" width="62.88671875" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="11" customWidth="1"/>
     <col min="9" max="9" width="26" style="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -5481,7 +5512,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="C2" s="6"/>
       <c r="D2" s="7"/>
@@ -5491,27 +5522,27 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>404</v>
+        <v>395</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>70</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>405</v>
+        <v>396</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>54</v>
@@ -5520,24 +5551,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>33</v>
@@ -5549,24 +5580,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="100.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>197</v>
-      </c>
       <c r="C5" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>200</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>208</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>33</v>
@@ -5578,24 +5609,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="145.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>33</v>
@@ -5607,27 +5638,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="145.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="145.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>27</v>
@@ -5636,27 +5667,27 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="145.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>27</v>
@@ -5665,24 +5696,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="155.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="155.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>33</v>
@@ -5694,24 +5725,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="164.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="164.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>205</v>
-      </c>
       <c r="D10" s="7" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>33</v>
@@ -5723,27 +5754,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="193.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="193.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>324</v>
+        <v>315</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>27</v>
@@ -5752,24 +5783,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="110.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>33</v>
@@ -5791,20 +5822,20 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22796737-2425-43B9-A206-255239ECAB63}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="71.140625" customWidth="1"/>
-    <col min="5" max="5" width="40.85546875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="62.85546875" customWidth="1"/>
-    <col min="7" max="7" width="43.5703125" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="11" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="71.109375" customWidth="1"/>
+    <col min="5" max="5" width="40.88671875" style="11" customWidth="1"/>
+    <col min="6" max="6" width="62.88671875" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="11" customWidth="1"/>
     <col min="9" max="9" width="26" style="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -5833,7 +5864,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="D2" s="7"/>
       <c r="E2" s="5"/>
@@ -5842,24 +5873,24 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="145.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>247</v>
-      </c>
       <c r="F3" s="7" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>33</v>
@@ -5871,27 +5902,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="1" customFormat="1" ht="91.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="1" customFormat="1" ht="91.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>250</v>
-      </c>
       <c r="E4" s="5" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>27</v>
@@ -5900,24 +5931,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="106.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="106.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>239</v>
-      </c>
       <c r="C5" s="5" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>33</v>
@@ -5929,24 +5960,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="185.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="185.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>33</v>
@@ -5958,27 +5989,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="158.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>411</v>
+        <v>402</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>412</v>
+        <v>403</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>27</v>
@@ -5987,24 +6018,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="147" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="147" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="G8" s="7" t="s">
         <v>33</v>
@@ -6016,27 +6047,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="163.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="163.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>326</v>
+        <v>317</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>27</v>
@@ -6045,24 +6076,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="167.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="167.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>327</v>
+        <v>318</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>33</v>
@@ -6074,24 +6105,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="190.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="190.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>245</v>
-      </c>
       <c r="D11" s="7" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>33</v>
@@ -6103,27 +6134,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="173.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="173.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>246</v>
-      </c>
       <c r="D12" s="7" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>328</v>
+        <v>319</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>27</v>
@@ -6142,20 +6173,20 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61ED5D93-E2AB-40AC-8E95-1F3195C9E8A1}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="71.140625" customWidth="1"/>
-    <col min="5" max="5" width="40.85546875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="62.85546875" customWidth="1"/>
-    <col min="7" max="7" width="43.5703125" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="11" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="71.109375" customWidth="1"/>
+    <col min="5" max="5" width="40.88671875" style="11" customWidth="1"/>
+    <col min="6" max="6" width="62.88671875" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="11" customWidth="1"/>
     <col min="9" max="9" width="26" style="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -6184,7 +6215,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="D2" s="7"/>
       <c r="E2" s="5"/>
@@ -6193,24 +6224,24 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="167.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="167.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>33</v>
@@ -6222,27 +6253,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="1" customFormat="1" ht="148.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="1" customFormat="1" ht="148.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>421</v>
+        <v>412</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>27</v>
@@ -6251,24 +6282,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="156.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="156.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>282</v>
-      </c>
       <c r="C5" s="5" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>33</v>
@@ -6280,24 +6311,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="156" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="156" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>33</v>
@@ -6309,24 +6340,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="195" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="195" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>33</v>
@@ -6338,27 +6369,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="189" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="189" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>329</v>
+        <v>320</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>27</v>
@@ -6367,24 +6398,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="159" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="159" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>33</v>
@@ -6396,24 +6427,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="153.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="153.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>331</v>
+        <v>322</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>33</v>
@@ -6425,27 +6456,27 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="169.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>282</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>290</v>
-      </c>
       <c r="D11" s="7" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>27</v>
@@ -6454,24 +6485,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="191.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="191.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>332</v>
+        <v>323</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>33</v>

</xml_diff>

<commit_message>
TC_LF_008 commited with updated file
</commit_message>
<xml_diff>
--- a/manual_test_cases/Daraz_Manual_Test_Checklist.xlsx
+++ b/manual_test_cases/Daraz_Manual_Test_Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\Automation_project\Daraz_Website_Automation_Using_Playwright\manual_test_cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C7E2080-1E03-43DE-909A-F26F70C3A83B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA733744-78E1-402C-B456-F569362098D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{02469D76-9D46-4AA2-AC21-F8D260897AAE}"/>
   </bookViews>
@@ -4673,32 +4673,32 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="126.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:9" s="29" customFormat="1" ht="126.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="25" t="s">
         <v>432</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="26" t="s">
         <v>435</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="24" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>

<commit_message>
TC_LG_003, TC_LG_004, TC_LG_005 updated
</commit_message>
<xml_diff>
--- a/manual_test_cases/Daraz_Manual_Test_Checklist.xlsx
+++ b/manual_test_cases/Daraz_Manual_Test_Checklist.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shifa\OneDrive\Documents\Automation_Projects\Daraz_Website_Automation_Using_Playwright\manual_test_cases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\Automation_project\Daraz_Website_Automation_Using_Playwright\manual_test_cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB946CB5-AC8F-4E5B-836E-0325B0025975}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF5F887-10E0-43BF-A13A-9D36B6FE6701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-12675" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{02469D76-9D46-4AA2-AC21-F8D260897AAE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{02469D76-9D46-4AA2-AC21-F8D260897AAE}"/>
   </bookViews>
   <sheets>
     <sheet name="Version History" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="437">
   <si>
     <t>Project Name :</t>
   </si>
@@ -2771,12 +2771,6 @@
     <t>Validate Logging out by selecting Logout option  from 'My Account' dropdown menu</t>
   </si>
   <si>
-    <t>Validate logging out and browsing back</t>
-  </si>
-  <si>
-    <t>Validate logout option is not displayed under 'My Account' dropmenu before logging in</t>
-  </si>
-  <si>
     <t>Validate logging out and logging in immediately</t>
   </si>
   <si>
@@ -2799,13 +2793,19 @@
   </si>
   <si>
     <t>After logging in, if the user closes the browser without logging out, the system should automatically log the user out. On reopening the application, the user should be required to log in again.</t>
+  </si>
+  <si>
+    <t>Validate user remains logged out after clicking browser back button</t>
+  </si>
+  <si>
+    <t>Validate logout option is not displayed before logging in</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2896,13 +2896,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF11734B"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -2966,7 +2959,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2993,9 +2986,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3040,7 +3030,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -3062,6 +3051,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3387,65 +3379,65 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1122DB24-336C-4BDE-AAFD-8F064C42F5B9}">
   <dimension ref="G1:U7"/>
-  <sheetFormatPr defaultRowHeight="26.25" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="25.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="7" max="7" width="45.85546875" style="17" customWidth="1"/>
-    <col min="8" max="8" width="2.140625" customWidth="1"/>
-    <col min="9" max="9" width="45.85546875" style="14" customWidth="1"/>
+    <col min="7" max="7" width="45.88671875" style="16" customWidth="1"/>
+    <col min="8" max="8" width="2.109375" customWidth="1"/>
+    <col min="9" max="9" width="45.88671875" style="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="7:21" ht="23.45" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="7:21" ht="60.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="G2" s="18" t="s">
+    <row r="1" spans="7:21" ht="23.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="7:21" ht="60.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="G2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="H2" s="16"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="20"/>
-      <c r="T2" s="20"/>
-      <c r="U2" s="20"/>
-    </row>
-    <row r="3" spans="7:21" ht="60" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="G3" s="18" t="s">
+      <c r="O2" s="18"/>
+      <c r="P2" s="18"/>
+      <c r="Q2" s="18"/>
+      <c r="R2" s="18"/>
+      <c r="S2" s="19"/>
+      <c r="T2" s="19"/>
+      <c r="U2" s="19"/>
+    </row>
+    <row r="3" spans="7:21" ht="60" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="G3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="16"/>
-      <c r="I3" s="22" t="s">
+      <c r="H3" s="15"/>
+      <c r="I3" s="21" t="s">
         <v>407</v>
       </c>
-      <c r="O3" s="19"/>
-      <c r="P3" s="19"/>
-      <c r="Q3" s="19"/>
-      <c r="R3" s="19"/>
-      <c r="S3" s="20"/>
-      <c r="T3" s="20"/>
-      <c r="U3" s="20"/>
-    </row>
-    <row r="4" spans="7:21" ht="60.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="G4" s="18" t="s">
+      <c r="O3" s="18"/>
+      <c r="P3" s="18"/>
+      <c r="Q3" s="18"/>
+      <c r="R3" s="18"/>
+      <c r="S3" s="19"/>
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+    </row>
+    <row r="4" spans="7:21" ht="60.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="G4" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="16"/>
-      <c r="I4" s="15" t="s">
+      <c r="H4" s="15"/>
+      <c r="I4" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
-      <c r="S4" s="20"/>
-      <c r="T4" s="20"/>
-      <c r="U4" s="20"/>
-    </row>
-    <row r="5" spans="7:21" ht="44.45" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="7:21" ht="55.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="7:21" ht="55.9" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="O4" s="18"/>
+      <c r="P4" s="18"/>
+      <c r="Q4" s="18"/>
+      <c r="R4" s="18"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+    </row>
+    <row r="5" spans="7:21" ht="44.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="7:21" ht="55.2" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="7:21" ht="55.95" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3455,19 +3447,19 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0792B093-2DBC-41B2-A40D-647FCC4C9792}">
   <dimension ref="A1:J16"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="2" width="20.85546875" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" customWidth="1"/>
-    <col min="4" max="4" width="40.85546875" style="11" customWidth="1"/>
-    <col min="5" max="5" width="71.140625" customWidth="1"/>
-    <col min="6" max="6" width="48.140625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="57.42578125" customWidth="1"/>
-    <col min="8" max="8" width="51.5703125" customWidth="1"/>
-    <col min="9" max="10" width="25.7109375" style="11" customWidth="1"/>
+    <col min="1" max="2" width="20.88671875" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" customWidth="1"/>
+    <col min="4" max="4" width="40.88671875" style="10" customWidth="1"/>
+    <col min="5" max="5" width="71.109375" customWidth="1"/>
+    <col min="6" max="6" width="48.109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="57.44140625" customWidth="1"/>
+    <col min="8" max="8" width="51.5546875" customWidth="1"/>
+    <col min="9" max="10" width="25.6640625" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>317</v>
       </c>
@@ -3499,7 +3491,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="6"/>
@@ -3510,7 +3502,7 @@
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
     </row>
-    <row r="3" spans="1:10" ht="152.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="152.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>322</v>
       </c>
@@ -3542,7 +3534,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="1" customFormat="1" ht="143.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" s="1" customFormat="1" ht="143.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>323</v>
       </c>
@@ -3574,7 +3566,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="155.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="155.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>324</v>
       </c>
@@ -3606,7 +3598,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="139.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="139.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>325</v>
       </c>
@@ -3638,7 +3630,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="159" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="159" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>326</v>
       </c>
@@ -3670,7 +3662,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>327</v>
       </c>
@@ -3702,7 +3694,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="168.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="168.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>328</v>
       </c>
@@ -3734,7 +3726,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="193.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="193.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>329</v>
       </c>
@@ -3766,7 +3758,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>330</v>
       </c>
@@ -3798,7 +3790,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="256.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="256.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>331</v>
       </c>
@@ -3830,7 +3822,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="270" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="270" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>332</v>
       </c>
@@ -3862,7 +3854,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="264.60000000000002" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="264.60000000000002" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>333</v>
       </c>
@@ -3894,7 +3886,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="292.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="292.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>334</v>
       </c>
@@ -3926,7 +3918,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="271.89999999999998" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="271.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>335</v>
       </c>
@@ -3968,21 +3960,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{160DC5CE-D4D6-45E5-9673-C5134C0EE041}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
-    <col min="3" max="3" width="45.85546875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="70.85546875" style="7" customWidth="1"/>
-    <col min="5" max="5" width="48.140625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="70.7109375" style="7" customWidth="1"/>
-    <col min="7" max="7" width="71.5703125" style="7" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="4" customWidth="1"/>
+    <col min="1" max="1" width="21.44140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" customWidth="1"/>
+    <col min="3" max="3" width="45.88671875" style="6" customWidth="1"/>
+    <col min="4" max="4" width="70.88671875" style="7" customWidth="1"/>
+    <col min="5" max="5" width="48.109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="70.6640625" style="7" customWidth="1"/>
+    <col min="7" max="7" width="71.5546875" style="7" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="4" customWidth="1"/>
     <col min="9" max="9" width="26" style="4" customWidth="1"/>
-    <col min="10" max="10" width="14.85546875" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -4011,33 +4003,35 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="29" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+    <row r="3" spans="1:10" s="27" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="22" t="s">
         <v>403</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="23" t="s">
         <v>402</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="24" t="s">
         <v>404</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="25" t="s">
         <v>399</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="24" t="s">
         <v>400</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="25" t="s">
         <v>401</v>
       </c>
-      <c r="G3" s="26" t="s">
+      <c r="G3" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="I3" s="27"/>
-      <c r="J3" s="28"/>
+      <c r="I3" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" s="26"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4048,20 +4042,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{126F3227-500D-408C-A3D2-9A52BE2F4C8C}">
   <dimension ref="A1:I31"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
-    <col min="3" max="3" width="45.85546875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="70.85546875" style="7" customWidth="1"/>
-    <col min="5" max="5" width="48.140625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="70.7109375" style="7" customWidth="1"/>
-    <col min="7" max="7" width="71.5703125" style="7" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="4" customWidth="1"/>
+    <col min="1" max="1" width="21.44140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" customWidth="1"/>
+    <col min="3" max="3" width="45.88671875" style="6" customWidth="1"/>
+    <col min="4" max="4" width="70.88671875" style="7" customWidth="1"/>
+    <col min="5" max="5" width="48.109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="70.6640625" style="7" customWidth="1"/>
+    <col min="7" max="7" width="71.5546875" style="7" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="4" customWidth="1"/>
     <col min="9" max="9" width="26" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -4090,7 +4084,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="156.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="156.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
@@ -4115,11 +4109,11 @@
       <c r="H3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="1" customFormat="1" ht="150" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="1" customFormat="1" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
@@ -4144,11 +4138,11 @@
       <c r="H4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="154.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="154.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
@@ -4173,11 +4167,11 @@
       <c r="H5" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I5" s="13" t="s">
+      <c r="I5" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="117.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="117.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
@@ -4202,11 +4196,11 @@
       <c r="H6" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="I6" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="157.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="157.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>13</v>
       </c>
@@ -4231,11 +4225,11 @@
       <c r="H7" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="I7" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="165" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="165" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
@@ -4260,11 +4254,11 @@
       <c r="H8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="128.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="128.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>15</v>
       </c>
@@ -4289,11 +4283,11 @@
       <c r="H9" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="I9" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="178.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="178.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>16</v>
       </c>
@@ -4318,11 +4312,11 @@
       <c r="H10" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="165.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="165.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>17</v>
       </c>
@@ -4347,11 +4341,11 @@
       <c r="H11" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="I11" s="13" t="s">
+      <c r="I11" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="120.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="120.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>18</v>
       </c>
@@ -4376,11 +4370,11 @@
       <c r="H12" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="I12" s="12" t="s">
+      <c r="I12" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="120.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="120.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>18</v>
       </c>
@@ -4405,30 +4399,30 @@
       <c r="H13" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="I13" s="12" t="s">
+      <c r="I13" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C25" s="21"/>
-    </row>
-    <row r="26" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C26" s="21"/>
-    </row>
-    <row r="27" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C27" s="21"/>
-    </row>
-    <row r="28" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C28" s="21"/>
-    </row>
-    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C29" s="21"/>
-    </row>
-    <row r="30" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C30" s="21"/>
-    </row>
-    <row r="31" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C31" s="21"/>
+    <row r="25" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C25" s="20"/>
+    </row>
+    <row r="26" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C26" s="20"/>
+    </row>
+    <row r="27" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C27" s="20"/>
+    </row>
+    <row r="28" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C28" s="20"/>
+    </row>
+    <row r="29" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C29" s="20"/>
+    </row>
+    <row r="30" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C30" s="20"/>
+    </row>
+    <row r="31" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C31" s="20"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
@@ -4440,20 +4434,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E58948E-B793-4546-A904-38FBA4A9768B}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" customWidth="1"/>
-    <col min="4" max="4" width="71.140625" customWidth="1"/>
-    <col min="5" max="5" width="40.85546875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="62.85546875" customWidth="1"/>
-    <col min="7" max="7" width="43.5703125" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="11" customWidth="1"/>
-    <col min="9" max="9" width="26" style="11" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" customWidth="1"/>
+    <col min="4" max="4" width="71.109375" customWidth="1"/>
+    <col min="5" max="5" width="40.88671875" style="10" customWidth="1"/>
+    <col min="6" max="6" width="62.88671875" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="10" customWidth="1"/>
+    <col min="9" max="9" width="26" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -4482,7 +4476,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="C2" s="6"/>
       <c r="D2" s="7"/>
@@ -4492,293 +4486,293 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" s="29" customFormat="1" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+    <row r="3" spans="1:9" s="27" customFormat="1" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="24" t="s">
         <v>405</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="G3" s="26" t="s">
+      <c r="G3" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="24" t="s">
+      <c r="I3" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="30" customFormat="1" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+    <row r="4" spans="1:9" s="28" customFormat="1" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="C4" s="24" t="s">
         <v>406</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="E4" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="G4" s="26" t="s">
+      <c r="G4" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="H4" s="24" t="s">
+      <c r="H4" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="24" t="s">
+      <c r="I4" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:9" s="29" customFormat="1" ht="105.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="23" t="s">
+    <row r="5" spans="1:9" s="27" customFormat="1" ht="105.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="24" t="s">
         <v>416</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="25" t="s">
         <v>408</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="24" t="s">
         <v>409</v>
       </c>
-      <c r="F5" s="26" t="s">
+      <c r="F5" s="25" t="s">
         <v>410</v>
       </c>
-      <c r="G5" s="26" t="s">
+      <c r="G5" s="25" t="s">
         <v>71</v>
       </c>
-      <c r="H5" s="24" t="s">
+      <c r="H5" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="I5" s="24" t="s">
+      <c r="I5" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:9" s="29" customFormat="1" ht="109.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="23" t="s">
+    <row r="6" spans="1:9" s="27" customFormat="1" ht="109.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="24" t="s">
         <v>417</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="25" t="s">
         <v>411</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="24" t="s">
         <v>350</v>
       </c>
-      <c r="F6" s="26" t="s">
+      <c r="F6" s="25" t="s">
         <v>410</v>
       </c>
-      <c r="G6" s="26" t="s">
+      <c r="G6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="H6" s="24" t="s">
+      <c r="H6" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="I6" s="24" t="s">
+      <c r="I6" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:9" s="29" customFormat="1" ht="136.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="23" t="s">
+    <row r="7" spans="1:9" s="27" customFormat="1" ht="136.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="24" t="s">
         <v>418</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="25" t="s">
         <v>412</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="24" t="s">
         <v>413</v>
       </c>
-      <c r="F7" s="26" t="s">
+      <c r="F7" s="25" t="s">
         <v>410</v>
       </c>
-      <c r="G7" s="26" t="s">
+      <c r="G7" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="H7" s="24" t="s">
+      <c r="H7" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="I7" s="24" t="s">
+      <c r="I7" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:9" s="29" customFormat="1" ht="118.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="23" t="s">
+    <row r="8" spans="1:9" s="27" customFormat="1" ht="118.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="24" t="s">
         <v>419</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="E8" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="F8" s="25" t="s">
         <v>414</v>
       </c>
-      <c r="G8" s="26" t="s">
+      <c r="G8" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="H8" s="24" t="s">
+      <c r="H8" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="I8" s="24" t="s">
+      <c r="I8" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:9" s="29" customFormat="1" ht="116.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="23" t="s">
+    <row r="9" spans="1:9" s="27" customFormat="1" ht="116.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="C9" s="24" t="s">
         <v>420</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="25" t="s">
         <v>415</v>
       </c>
-      <c r="E9" s="25" t="s">
+      <c r="E9" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="F9" s="31" t="s">
+      <c r="F9" s="29" t="s">
         <v>295</v>
       </c>
-      <c r="G9" s="31" t="s">
+      <c r="G9" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="24" t="s">
+      <c r="H9" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="I9" s="24" t="s">
+      <c r="I9" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:9" s="29" customFormat="1" ht="126.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="23" t="s">
+    <row r="10" spans="1:9" s="27" customFormat="1" ht="126.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="24" t="s">
         <v>421</v>
       </c>
-      <c r="D10" s="26" t="s">
+      <c r="D10" s="25" t="s">
         <v>424</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="F10" s="26" t="s">
+      <c r="F10" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="G10" s="26" t="s">
+      <c r="G10" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="H10" s="24" t="s">
+      <c r="H10" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="I10" s="24" t="s">
+      <c r="I10" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:9" s="36" customFormat="1" ht="125.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="32" t="s">
+    <row r="11" spans="1:9" s="34" customFormat="1" ht="125.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="30" t="s">
         <v>64</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="31" t="s">
         <v>55</v>
       </c>
-      <c r="C11" s="34" t="s">
+      <c r="C11" s="32" t="s">
         <v>422</v>
       </c>
-      <c r="D11" s="35" t="s">
+      <c r="D11" s="33" t="s">
         <v>81</v>
       </c>
-      <c r="E11" s="34" t="s">
+      <c r="E11" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="F11" s="35" t="s">
+      <c r="F11" s="33" t="s">
         <v>88</v>
       </c>
-      <c r="G11" s="35" t="s">
+      <c r="G11" s="33" t="s">
         <v>82</v>
       </c>
-      <c r="H11" s="33" t="s">
+      <c r="H11" s="31" t="s">
         <v>53</v>
       </c>
-      <c r="I11" s="33" t="s">
+      <c r="I11" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:9" s="29" customFormat="1" ht="140.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="23" t="s">
+    <row r="12" spans="1:9" s="27" customFormat="1" ht="140.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="24" t="s">
         <v>423</v>
       </c>
-      <c r="D12" s="26" t="s">
+      <c r="D12" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="E12" s="25" t="s">
+      <c r="E12" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="F12" s="26" t="s">
+      <c r="F12" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="G12" s="26" t="s">
+      <c r="G12" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="H12" s="24" t="s">
+      <c r="H12" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="I12" s="24" t="s">
+      <c r="I12" s="11" t="s">
         <v>23</v>
       </c>
     </row>
@@ -4792,20 +4786,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B70680C-BD57-41BD-B550-973B32609FA9}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" customWidth="1"/>
-    <col min="4" max="4" width="71.140625" customWidth="1"/>
-    <col min="5" max="5" width="40.85546875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="62.85546875" customWidth="1"/>
-    <col min="7" max="7" width="43.5703125" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="11" customWidth="1"/>
-    <col min="9" max="9" width="26" style="11" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" customWidth="1"/>
+    <col min="4" max="4" width="71.109375" customWidth="1"/>
+    <col min="5" max="5" width="40.88671875" style="10" customWidth="1"/>
+    <col min="6" max="6" width="62.88671875" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="10" customWidth="1"/>
+    <col min="9" max="9" width="26" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -4834,7 +4828,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="C2" s="6"/>
       <c r="D2" s="7"/>
@@ -4844,152 +4838,152 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" s="29" customFormat="1" ht="100.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+    <row r="3" spans="1:9" s="27" customFormat="1" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="24" t="s">
         <v>426</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="25" t="s">
         <v>105</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="G3" s="26" t="s">
+      <c r="G3" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="24" t="s">
+      <c r="I3" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="30" customFormat="1" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+    <row r="4" spans="1:9" s="28" customFormat="1" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="C4" s="24" t="s">
+        <v>433</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="E4" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="F4" s="25" t="s">
+        <v>434</v>
+      </c>
+      <c r="G4" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="H4" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="27" customFormat="1" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="24" t="s">
         <v>435</v>
       </c>
-      <c r="D4" s="26" t="s">
-        <v>101</v>
-      </c>
-      <c r="E4" s="25" t="s">
+      <c r="D5" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="E5" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F5" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="G5" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="27" customFormat="1" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="C6" s="24" t="s">
         <v>436</v>
       </c>
-      <c r="G4" s="26" t="s">
-        <v>102</v>
-      </c>
-      <c r="H4" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" s="24" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="100.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B5" s="4" t="s">
+      <c r="D6" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="E6" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" s="35" t="s">
+        <v>107</v>
+      </c>
+      <c r="G6" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" s="27" customFormat="1" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C7" s="24" t="s">
         <v>427</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="E5" s="5" t="s">
+      <c r="D7" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="E7" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="G5" s="7" t="s">
+      <c r="F7" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="G7" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="H5" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" s="12" t="s">
+      <c r="H7" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>428</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I6" s="12" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="100.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>429</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="I7" s="12" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>94</v>
       </c>
@@ -4997,7 +4991,7 @@
         <v>99</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>110</v>
@@ -5014,11 +5008,11 @@
       <c r="H8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="I8" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>96</v>
       </c>
@@ -5026,7 +5020,7 @@
         <v>99</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>110</v>
@@ -5043,11 +5037,11 @@
       <c r="H9" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="I9" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>95</v>
       </c>
@@ -5055,7 +5049,7 @@
         <v>99</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>110</v>
@@ -5072,11 +5066,11 @@
       <c r="H10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I10" s="13" t="s">
+      <c r="I10" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>97</v>
       </c>
@@ -5084,7 +5078,7 @@
         <v>99</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>110</v>
@@ -5099,13 +5093,13 @@
         <v>32</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="I11" s="12" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="131.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="131.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>98</v>
       </c>
@@ -5113,7 +5107,7 @@
         <v>99</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>161</v>
@@ -5130,7 +5124,7 @@
       <c r="H12" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="I12" s="12" t="s">
+      <c r="I12" s="11" t="s">
         <v>23</v>
       </c>
     </row>
@@ -5144,20 +5138,20 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0658FF2-697D-4C69-B42D-CDE2007A7D77}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" customWidth="1"/>
-    <col min="4" max="4" width="71.140625" customWidth="1"/>
-    <col min="5" max="5" width="40.85546875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="62.85546875" customWidth="1"/>
-    <col min="7" max="7" width="43.5703125" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="11" customWidth="1"/>
-    <col min="9" max="9" width="26" style="11" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" customWidth="1"/>
+    <col min="4" max="4" width="71.109375" customWidth="1"/>
+    <col min="5" max="5" width="40.88671875" style="10" customWidth="1"/>
+    <col min="6" max="6" width="62.88671875" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="10" customWidth="1"/>
+    <col min="9" max="9" width="26" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -5186,7 +5180,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="C2" s="6"/>
       <c r="D2" s="7"/>
@@ -5196,7 +5190,7 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>119</v>
       </c>
@@ -5221,11 +5215,11 @@
       <c r="H3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="1" customFormat="1" ht="90.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="1" customFormat="1" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>120</v>
       </c>
@@ -5250,11 +5244,11 @@
       <c r="H4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>121</v>
       </c>
@@ -5279,11 +5273,11 @@
       <c r="H5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I5" s="12" t="s">
+      <c r="I5" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>122</v>
       </c>
@@ -5308,11 +5302,11 @@
       <c r="H6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I6" s="13" t="s">
+      <c r="I6" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>123</v>
       </c>
@@ -5337,11 +5331,11 @@
       <c r="H7" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="I7" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>124</v>
       </c>
@@ -5366,11 +5360,11 @@
       <c r="H8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="91.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="91.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>125</v>
       </c>
@@ -5395,11 +5389,11 @@
       <c r="H9" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="12" t="s">
+      <c r="I9" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="150" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>126</v>
       </c>
@@ -5424,11 +5418,11 @@
       <c r="H10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>127</v>
       </c>
@@ -5453,11 +5447,11 @@
       <c r="H11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I11" s="12" t="s">
+      <c r="I11" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>128</v>
       </c>
@@ -5482,7 +5476,7 @@
       <c r="H12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I12" s="13" t="s">
+      <c r="I12" s="12" t="s">
         <v>27</v>
       </c>
     </row>
@@ -5496,20 +5490,20 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B3B9881-CF40-4798-A105-6C45CF8840BD}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" customWidth="1"/>
-    <col min="4" max="4" width="71.140625" customWidth="1"/>
-    <col min="5" max="5" width="40.85546875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="62.85546875" customWidth="1"/>
-    <col min="7" max="7" width="43.5703125" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="11" customWidth="1"/>
-    <col min="9" max="9" width="26" style="11" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" customWidth="1"/>
+    <col min="4" max="4" width="71.109375" customWidth="1"/>
+    <col min="5" max="5" width="40.88671875" style="10" customWidth="1"/>
+    <col min="6" max="6" width="62.88671875" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="10" customWidth="1"/>
+    <col min="9" max="9" width="26" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -5538,7 +5532,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="C2" s="6"/>
       <c r="D2" s="7"/>
@@ -5548,7 +5542,7 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>162</v>
       </c>
@@ -5573,11 +5567,11 @@
       <c r="H3" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="I3" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>163</v>
       </c>
@@ -5602,11 +5596,11 @@
       <c r="H4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="100.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>164</v>
       </c>
@@ -5631,11 +5625,11 @@
       <c r="H5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I5" s="12" t="s">
+      <c r="I5" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="145.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>165</v>
       </c>
@@ -5660,11 +5654,11 @@
       <c r="H6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="I6" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="145.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="145.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>166</v>
       </c>
@@ -5689,11 +5683,11 @@
       <c r="H7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="13" t="s">
+      <c r="I7" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="145.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>167</v>
       </c>
@@ -5718,11 +5712,11 @@
       <c r="H8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="155.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="155.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>168</v>
       </c>
@@ -5747,11 +5741,11 @@
       <c r="H9" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="12" t="s">
+      <c r="I9" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="164.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="164.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>169</v>
       </c>
@@ -5776,11 +5770,11 @@
       <c r="H10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="193.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="193.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>170</v>
       </c>
@@ -5805,11 +5799,11 @@
       <c r="H11" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I11" s="13" t="s">
+      <c r="I11" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="110.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>171</v>
       </c>
@@ -5834,7 +5828,7 @@
       <c r="H12" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I12" s="12" t="s">
+      <c r="I12" s="11" t="s">
         <v>23</v>
       </c>
     </row>
@@ -5848,20 +5842,20 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22796737-2425-43B9-A206-255239ECAB63}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="71.140625" customWidth="1"/>
-    <col min="5" max="5" width="40.85546875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="62.85546875" customWidth="1"/>
-    <col min="7" max="7" width="43.5703125" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="11" customWidth="1"/>
-    <col min="9" max="9" width="26" style="11" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="71.109375" customWidth="1"/>
+    <col min="5" max="5" width="40.88671875" style="10" customWidth="1"/>
+    <col min="6" max="6" width="62.88671875" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="10" customWidth="1"/>
+    <col min="9" max="9" width="26" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -5890,7 +5884,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="D2" s="7"/>
       <c r="E2" s="5"/>
@@ -5899,7 +5893,7 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="145.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>204</v>
       </c>
@@ -5924,11 +5918,11 @@
       <c r="H3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="1" customFormat="1" ht="91.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="1" customFormat="1" ht="91.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>205</v>
       </c>
@@ -5953,11 +5947,11 @@
       <c r="H4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="106.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="106.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>206</v>
       </c>
@@ -5982,11 +5976,11 @@
       <c r="H5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I5" s="12" t="s">
+      <c r="I5" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="185.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="185.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>207</v>
       </c>
@@ -6011,11 +6005,11 @@
       <c r="H6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="I6" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="158.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>208</v>
       </c>
@@ -6040,11 +6034,11 @@
       <c r="H7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="13" t="s">
+      <c r="I7" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="147" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="147" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>209</v>
       </c>
@@ -6069,11 +6063,11 @@
       <c r="H8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="I8" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="163.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="163.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>210</v>
       </c>
@@ -6098,11 +6092,11 @@
       <c r="H9" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="I9" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="167.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="167.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>211</v>
       </c>
@@ -6127,11 +6121,11 @@
       <c r="H10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="190.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="190.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>212</v>
       </c>
@@ -6156,11 +6150,11 @@
       <c r="H11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I11" s="12" t="s">
+      <c r="I11" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="173.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="173.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>213</v>
       </c>
@@ -6185,7 +6179,7 @@
       <c r="H12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I12" s="13" t="s">
+      <c r="I12" s="12" t="s">
         <v>27</v>
       </c>
     </row>
@@ -6199,20 +6193,20 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61ED5D93-E2AB-40AC-8E95-1F3195C9E8A1}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="71.140625" customWidth="1"/>
-    <col min="5" max="5" width="40.85546875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="62.85546875" customWidth="1"/>
-    <col min="7" max="7" width="43.5703125" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="11" customWidth="1"/>
-    <col min="9" max="9" width="26" style="11" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="71.109375" customWidth="1"/>
+    <col min="5" max="5" width="40.88671875" style="10" customWidth="1"/>
+    <col min="6" max="6" width="62.88671875" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" style="10" customWidth="1"/>
+    <col min="9" max="9" width="26" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -6241,7 +6235,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="D2" s="7"/>
       <c r="E2" s="5"/>
@@ -6250,7 +6244,7 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="167.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="167.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>247</v>
       </c>
@@ -6275,11 +6269,11 @@
       <c r="H3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="1" customFormat="1" ht="148.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="1" customFormat="1" ht="148.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>248</v>
       </c>
@@ -6304,11 +6298,11 @@
       <c r="H4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="156.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="156.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>249</v>
       </c>
@@ -6333,11 +6327,11 @@
       <c r="H5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I5" s="12" t="s">
+      <c r="I5" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="156" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="156" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>250</v>
       </c>
@@ -6362,11 +6356,11 @@
       <c r="H6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="I6" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="195" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="195" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>251</v>
       </c>
@@ -6391,11 +6385,11 @@
       <c r="H7" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="I7" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="189" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="189" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>252</v>
       </c>
@@ -6420,11 +6414,11 @@
       <c r="H8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="159" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="159" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>253</v>
       </c>
@@ -6449,11 +6443,11 @@
       <c r="H9" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="12" t="s">
+      <c r="I9" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="153.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="153.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>254</v>
       </c>
@@ -6478,11 +6472,11 @@
       <c r="H10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="169.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>255</v>
       </c>
@@ -6507,11 +6501,11 @@
       <c r="H11" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I11" s="13" t="s">
+      <c r="I11" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="191.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="191.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>256</v>
       </c>
@@ -6536,7 +6530,7 @@
       <c r="H12" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I12" s="12" t="s">
+      <c r="I12" s="11" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>

<commit_message>
TC_SF_001 TC_SF_002 TC_SF_003 updated
</commit_message>
<xml_diff>
--- a/manual_test_cases/Daraz_Manual_Test_Checklist.xlsx
+++ b/manual_test_cases/Daraz_Manual_Test_Checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\Automation_project\Daraz_Website_Automation_Using_Playwright\manual_test_cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF5F887-10E0-43BF-A13A-9D36B6FE6701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E1A80B5-6603-447A-BC05-849A04F8B648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{02469D76-9D46-4AA2-AC21-F8D260897AAE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{02469D76-9D46-4AA2-AC21-F8D260897AAE}"/>
   </bookViews>
   <sheets>
     <sheet name="Version History" sheetId="1" r:id="rId1"/>
@@ -703,32 +703,11 @@
     <t>TC_SF_010</t>
   </si>
   <si>
-    <t>Verify that the search bar is visible on the homepage.</t>
-  </si>
-  <si>
-    <t>Validate searching with an existig product name.</t>
-  </si>
-  <si>
-    <t>Validate searching with a non existig product name.</t>
-  </si>
-  <si>
-    <t>Verify that clicking the search icon/button initiates the search.</t>
-  </si>
-  <si>
-    <t>Verify that clicking a product from the search results opens the product details page.</t>
-  </si>
-  <si>
-    <t>Verify that search results shows accurate products that match the search keyword.</t>
-  </si>
-  <si>
     <t>1) Login to the application providing valid credentials.
 2) Go to the Home page.
 3) Observe the top section of the homepage.</t>
   </si>
   <si>
-    <t>Verify that the search button is visible.</t>
-  </si>
-  <si>
     <t xml:space="preserve">A search button with appopiate icon should be visible at the right corner of the search bar. </t>
   </si>
   <si>
@@ -756,16 +735,10 @@
     <t>Some products are showing at the bottom which does not match with the search key word.</t>
   </si>
   <si>
-    <t>Validate searching using partial product name shows relevant results.</t>
-  </si>
-  <si>
     <t>Procuct name: Wat</t>
   </si>
   <si>
     <t xml:space="preserve">Searched product should be displayed in the search results. </t>
-  </si>
-  <si>
-    <t>Validate filter options (brand, price, color, size) are available and apply correctly to the search results.</t>
   </si>
   <si>
     <r>
@@ -808,9 +781,6 @@
   </si>
   <si>
     <t>Procuct name: Umbrella</t>
-  </si>
-  <si>
-    <t>Verify that search results are displayed within acceptable load time.</t>
   </si>
   <si>
     <t>After clicking search button it sould not take more than 3 seconds to show result.</t>
@@ -2799,6 +2769,36 @@
   </si>
   <si>
     <t>Validate logout option is not displayed before logging in</t>
+  </si>
+  <si>
+    <t>Verify that the search button is visible</t>
+  </si>
+  <si>
+    <t>Validate searching with an existig product name</t>
+  </si>
+  <si>
+    <t>Validate searching with a non existig product name</t>
+  </si>
+  <si>
+    <t>Verify that clicking the search icon/button initiates the search</t>
+  </si>
+  <si>
+    <t>Verify that search results shows accurate products that match the search keyword</t>
+  </si>
+  <si>
+    <t>Validate searching using partial product name shows relevant results</t>
+  </si>
+  <si>
+    <t>Validate filter options (brand, price, color, size) are available and apply correctly to the search results</t>
+  </si>
+  <si>
+    <t>Verify that clicking a product from the search results opens the product details page</t>
+  </si>
+  <si>
+    <t>Verify that search results are displayed within acceptable load time</t>
+  </si>
+  <si>
+    <t>Verify that the search box is visible on the homepage</t>
   </si>
 </sst>
 </file>
@@ -3393,7 +3393,7 @@
       </c>
       <c r="H2" s="15"/>
       <c r="I2" s="14" t="s">
-        <v>291</v>
+        <v>281</v>
       </c>
       <c r="O2" s="18"/>
       <c r="P2" s="18"/>
@@ -3409,7 +3409,7 @@
       </c>
       <c r="H3" s="15"/>
       <c r="I3" s="21" t="s">
-        <v>407</v>
+        <v>397</v>
       </c>
       <c r="O3" s="18"/>
       <c r="P3" s="18"/>
@@ -3425,7 +3425,7 @@
       </c>
       <c r="H4" s="15"/>
       <c r="I4" s="14" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
       <c r="O4" s="18"/>
       <c r="P4" s="18"/>
@@ -3461,19 +3461,19 @@
   <sheetData>
     <row r="1" spans="1:10" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>66</v>
@@ -3485,10 +3485,10 @@
         <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>321</v>
+        <v>311</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -3504,54 +3504,54 @@
     </row>
     <row r="3" spans="1:10" ht="152.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>322</v>
+        <v>312</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>337</v>
+        <v>327</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>338</v>
+        <v>328</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>344</v>
+        <v>334</v>
       </c>
       <c r="H3" s="7" t="s">
         <v>33</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>342</v>
+        <v>332</v>
       </c>
     </row>
     <row r="4" spans="1:10" s="1" customFormat="1" ht="143.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>323</v>
+        <v>313</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>345</v>
+        <v>335</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>346</v>
+        <v>336</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>74</v>
@@ -3560,394 +3560,394 @@
         <v>39</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>342</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="155.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>58</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>347</v>
+        <v>337</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>55</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>353</v>
+        <v>343</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>70</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
       <c r="H5" s="7" t="s">
         <v>71</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="139.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>325</v>
+        <v>315</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>59</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>349</v>
+        <v>339</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>55</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>352</v>
+        <v>342</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>355</v>
+        <v>345</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>77</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="159" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>326</v>
+        <v>316</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>90</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>351</v>
+        <v>341</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>99</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>354</v>
+        <v>344</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>76</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>356</v>
+        <v>346</v>
       </c>
       <c r="H7" s="7" t="s">
         <v>102</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>357</v>
+        <v>347</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>358</v>
+        <v>348</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>327</v>
+        <v>317</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>95</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>359</v>
+        <v>349</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>99</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>360</v>
+        <v>350</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>76</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>362</v>
+        <v>352</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>357</v>
+        <v>347</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>358</v>
+        <v>348</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="168.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>328</v>
+        <v>318</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>120</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>363</v>
+        <v>353</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>118</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>364</v>
+        <v>354</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>76</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>365</v>
+        <v>355</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="193.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>128</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>366</v>
+        <v>356</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>118</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>373</v>
+        <v>363</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>374</v>
+        <v>364</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>375</v>
+        <v>365</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>357</v>
+        <v>347</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>376</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>172</v>
-      </c>
       <c r="E11" s="7" t="s">
-        <v>377</v>
+        <v>367</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>76</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>379</v>
+        <v>369</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>357</v>
+        <v>347</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>380</v>
+        <v>370</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="256.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>381</v>
+        <v>371</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>383</v>
+        <v>373</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>365</v>
+        <v>355</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="270" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>332</v>
+        <v>322</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>384</v>
+        <v>374</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>387</v>
+        <v>377</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>365</v>
+        <v>355</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="264.60000000000002" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>333</v>
+        <v>323</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>389</v>
+        <v>379</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>391</v>
+        <v>381</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="292.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>334</v>
+        <v>324</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>392</v>
+        <v>382</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>393</v>
+        <v>383</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>394</v>
+        <v>384</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>365</v>
+        <v>355</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="271.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>335</v>
+        <v>325</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>396</v>
+        <v>386</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>397</v>
+        <v>387</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>398</v>
+        <v>388</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>365</v>
+        <v>355</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
     </row>
   </sheetData>
@@ -4005,22 +4005,22 @@
     </row>
     <row r="3" spans="1:10" s="27" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>403</v>
+        <v>393</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>402</v>
+        <v>392</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>404</v>
+        <v>394</v>
       </c>
       <c r="D3" s="25" t="s">
-        <v>399</v>
+        <v>389</v>
       </c>
       <c r="E3" s="24" t="s">
-        <v>400</v>
+        <v>390</v>
       </c>
       <c r="F3" s="25" t="s">
-        <v>401</v>
+        <v>391</v>
       </c>
       <c r="G3" s="25" t="s">
         <v>32</v>
@@ -4092,13 +4092,13 @@
         <v>19</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>425</v>
+        <v>415</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>339</v>
+        <v>329</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>20</v>
@@ -4124,13 +4124,13 @@
         <v>25</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>343</v>
+        <v>333</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>33</v>
@@ -4153,10 +4153,10 @@
         <v>28</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>72</v>
@@ -4185,7 +4185,7 @@
         <v>30</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>31</v>
@@ -4214,7 +4214,7 @@
         <v>37</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>73</v>
@@ -4243,7 +4243,7 @@
         <v>38</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>74</v>
@@ -4272,7 +4272,7 @@
         <v>42</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="F9" s="7" t="s">
         <v>43</v>
@@ -4301,7 +4301,7 @@
         <v>45</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>46</v>
@@ -4330,7 +4330,7 @@
         <v>49</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>75</v>
@@ -4359,7 +4359,7 @@
         <v>51</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>52</v>
@@ -4388,7 +4388,7 @@
         <v>51</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>52</v>
@@ -4494,7 +4494,7 @@
         <v>55</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>405</v>
+        <v>395</v>
       </c>
       <c r="D3" s="25" t="s">
         <v>79</v>
@@ -4523,7 +4523,7 @@
         <v>55</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>406</v>
+        <v>396</v>
       </c>
       <c r="D4" s="25" t="s">
         <v>85</v>
@@ -4552,16 +4552,16 @@
         <v>55</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>416</v>
+        <v>406</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>408</v>
+        <v>398</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>409</v>
+        <v>399</v>
       </c>
       <c r="F5" s="25" t="s">
-        <v>410</v>
+        <v>400</v>
       </c>
       <c r="G5" s="25" t="s">
         <v>71</v>
@@ -4581,16 +4581,16 @@
         <v>55</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>417</v>
+        <v>407</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>411</v>
+        <v>401</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>350</v>
+        <v>340</v>
       </c>
       <c r="F6" s="25" t="s">
-        <v>410</v>
+        <v>400</v>
       </c>
       <c r="G6" s="25" t="s">
         <v>77</v>
@@ -4610,16 +4610,16 @@
         <v>55</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>418</v>
+        <v>408</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>412</v>
+        <v>402</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>413</v>
+        <v>403</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>410</v>
+        <v>400</v>
       </c>
       <c r="G7" s="25" t="s">
         <v>32</v>
@@ -4639,7 +4639,7 @@
         <v>55</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>419</v>
+        <v>409</v>
       </c>
       <c r="D8" s="25" t="s">
         <v>86</v>
@@ -4648,7 +4648,7 @@
         <v>78</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>414</v>
+        <v>404</v>
       </c>
       <c r="G8" s="25" t="s">
         <v>32</v>
@@ -4668,16 +4668,16 @@
         <v>55</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>415</v>
+        <v>405</v>
       </c>
       <c r="E9" s="24" t="s">
         <v>78</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="G9" s="29" t="s">
         <v>87</v>
@@ -4697,10 +4697,10 @@
         <v>55</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>421</v>
+        <v>411</v>
       </c>
       <c r="D10" s="25" t="s">
-        <v>424</v>
+        <v>414</v>
       </c>
       <c r="E10" s="24" t="s">
         <v>76</v>
@@ -4726,7 +4726,7 @@
         <v>55</v>
       </c>
       <c r="C11" s="32" t="s">
-        <v>422</v>
+        <v>412</v>
       </c>
       <c r="D11" s="33" t="s">
         <v>81</v>
@@ -4755,7 +4755,7 @@
         <v>55</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>423</v>
+        <v>413</v>
       </c>
       <c r="D12" s="25" t="s">
         <v>83</v>
@@ -4846,7 +4846,7 @@
         <v>99</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>426</v>
+        <v>416</v>
       </c>
       <c r="D3" s="25" t="s">
         <v>105</v>
@@ -4875,7 +4875,7 @@
         <v>99</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>433</v>
+        <v>423</v>
       </c>
       <c r="D4" s="25" t="s">
         <v>101</v>
@@ -4884,7 +4884,7 @@
         <v>78</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>434</v>
+        <v>424</v>
       </c>
       <c r="G4" s="25" t="s">
         <v>102</v>
@@ -4904,7 +4904,7 @@
         <v>99</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>435</v>
+        <v>425</v>
       </c>
       <c r="D5" s="25" t="s">
         <v>106</v>
@@ -4933,7 +4933,7 @@
         <v>99</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>436</v>
+        <v>426</v>
       </c>
       <c r="D6" s="25" t="s">
         <v>104</v>
@@ -4962,7 +4962,7 @@
         <v>99</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>427</v>
+        <v>417</v>
       </c>
       <c r="D7" s="25" t="s">
         <v>108</v>
@@ -4991,7 +4991,7 @@
         <v>99</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>428</v>
+        <v>418</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>110</v>
@@ -5020,7 +5020,7 @@
         <v>99</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>429</v>
+        <v>419</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>110</v>
@@ -5049,7 +5049,7 @@
         <v>99</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>110</v>
@@ -5078,7 +5078,7 @@
         <v>99</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>431</v>
+        <v>421</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>110</v>
@@ -5107,10 +5107,10 @@
         <v>99</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>432</v>
+        <v>422</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>78</v>
@@ -5190,87 +5190,87 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:9" s="27" customFormat="1" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="24" t="s">
+        <v>436</v>
+      </c>
+      <c r="D3" s="25" t="s">
         <v>129</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="F3" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="G3" s="7" t="s">
+      <c r="F3" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="G3" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="23" t="s">
         <v>21</v>
       </c>
       <c r="I3" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="1" customFormat="1" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:9" s="28" customFormat="1" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="E4" s="5" t="s">
+      <c r="C4" s="24" t="s">
+        <v>427</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="E4" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="F4" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="H4" s="4" t="s">
+      <c r="F4" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="G4" s="25" t="s">
+        <v>131</v>
+      </c>
+      <c r="H4" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="12" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="I4" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="27" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>367</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="G5" s="7" t="s">
+      <c r="C5" s="24" t="s">
+        <v>428</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>357</v>
+      </c>
+      <c r="E5" s="24" t="s">
+        <v>132</v>
+      </c>
+      <c r="F5" s="25" t="s">
+        <v>140</v>
+      </c>
+      <c r="G5" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="23" t="s">
         <v>21</v>
       </c>
       <c r="I5" s="11" t="s">
@@ -5285,19 +5285,19 @@
         <v>118</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>131</v>
+        <v>429</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>368</v>
+        <v>358</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>26</v>
@@ -5314,16 +5314,16 @@
         <v>118</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>132</v>
+        <v>430</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>367</v>
+        <v>357</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>32</v>
@@ -5343,19 +5343,19 @@
         <v>118</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>134</v>
+        <v>431</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>367</v>
+        <v>357</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>26</v>
@@ -5372,16 +5372,16 @@
         <v>118</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>146</v>
+        <v>432</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>369</v>
+        <v>359</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>32</v>
@@ -5401,16 +5401,16 @@
         <v>118</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>149</v>
+        <v>433</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>370</v>
+        <v>360</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>32</v>
@@ -5430,16 +5430,16 @@
         <v>118</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>133</v>
+        <v>434</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>371</v>
+        <v>361</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>32</v>
@@ -5459,19 +5459,19 @@
         <v>118</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>154</v>
+        <v>435</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>372</v>
+        <v>362</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>26</v>
@@ -5544,25 +5544,25 @@
     </row>
     <row r="3" spans="1:9" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>172</v>
-      </c>
       <c r="C3" s="5" t="s">
-        <v>378</v>
+        <v>368</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>379</v>
+        <v>369</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>53</v>
@@ -5573,22 +5573,22 @@
     </row>
     <row r="4" spans="1:9" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>184</v>
-      </c>
       <c r="E4" s="5" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>32</v>
@@ -5602,22 +5602,22 @@
     </row>
     <row r="5" spans="1:9" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>185</v>
-      </c>
       <c r="E5" s="5" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>32</v>
@@ -5631,22 +5631,22 @@
     </row>
     <row r="6" spans="1:9" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>186</v>
-      </c>
       <c r="E6" s="5" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>32</v>
@@ -5660,25 +5660,25 @@
     </row>
     <row r="7" spans="1:9" ht="145.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>26</v>
@@ -5689,25 +5689,25 @@
     </row>
     <row r="8" spans="1:9" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>26</v>
@@ -5718,22 +5718,22 @@
     </row>
     <row r="9" spans="1:9" ht="155.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>32</v>
@@ -5747,22 +5747,22 @@
     </row>
     <row r="10" spans="1:9" ht="164.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>32</v>
@@ -5776,25 +5776,25 @@
     </row>
     <row r="11" spans="1:9" ht="193.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>26</v>
@@ -5805,22 +5805,22 @@
     </row>
     <row r="12" spans="1:9" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>182</v>
-      </c>
       <c r="D12" s="7" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>32</v>
@@ -5895,22 +5895,22 @@
     </row>
     <row r="3" spans="1:9" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="F3" s="7" t="s">
         <v>214</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>223</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>224</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>32</v>
@@ -5924,25 +5924,25 @@
     </row>
     <row r="4" spans="1:9" s="1" customFormat="1" ht="91.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>26</v>
@@ -5953,22 +5953,22 @@
     </row>
     <row r="5" spans="1:9" ht="106.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>216</v>
-      </c>
       <c r="D5" s="7" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>32</v>
@@ -5982,22 +5982,22 @@
     </row>
     <row r="6" spans="1:9" ht="185.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>32</v>
@@ -6011,25 +6011,25 @@
     </row>
     <row r="7" spans="1:9" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>26</v>
@@ -6040,22 +6040,22 @@
     </row>
     <row r="8" spans="1:9" ht="147" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="G8" s="7" t="s">
         <v>32</v>
@@ -6069,25 +6069,25 @@
     </row>
     <row r="9" spans="1:9" ht="163.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>26</v>
@@ -6098,22 +6098,22 @@
     </row>
     <row r="10" spans="1:9" ht="167.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>301</v>
+        <v>291</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>32</v>
@@ -6127,22 +6127,22 @@
     </row>
     <row r="11" spans="1:9" ht="190.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>32</v>
@@ -6156,25 +6156,25 @@
     </row>
     <row r="12" spans="1:9" ht="173.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>26</v>
@@ -6246,22 +6246,22 @@
     </row>
     <row r="3" spans="1:9" ht="167.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>258</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>267</v>
-      </c>
       <c r="E3" s="5" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>32</v>
@@ -6275,25 +6275,25 @@
     </row>
     <row r="4" spans="1:9" s="1" customFormat="1" ht="148.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>395</v>
+        <v>385</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>26</v>
@@ -6304,22 +6304,22 @@
     </row>
     <row r="5" spans="1:9" ht="156.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>32</v>
@@ -6333,22 +6333,22 @@
     </row>
     <row r="6" spans="1:9" ht="156" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>275</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>271</v>
-      </c>
       <c r="F6" s="7" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>32</v>
@@ -6362,22 +6362,22 @@
     </row>
     <row r="7" spans="1:9" ht="195" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>277</v>
+        <v>267</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>32</v>
@@ -6391,25 +6391,25 @@
     </row>
     <row r="8" spans="1:9" ht="189" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>26</v>
@@ -6420,22 +6420,22 @@
     </row>
     <row r="9" spans="1:9" ht="159" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>32</v>
@@ -6449,22 +6449,22 @@
     </row>
     <row r="10" spans="1:9" ht="153.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>264</v>
-      </c>
       <c r="D10" s="7" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>305</v>
+        <v>295</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>32</v>
@@ -6478,25 +6478,25 @@
     </row>
     <row r="11" spans="1:9" ht="169.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>265</v>
-      </c>
       <c r="D11" s="7" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>26</v>
@@ -6507,22 +6507,22 @@
     </row>
     <row r="12" spans="1:9" ht="191.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>266</v>
-      </c>
       <c r="D12" s="7" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>306</v>
+        <v>296</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>32</v>

</xml_diff>